<commit_message>
huge update but 1 to 7 widget done and sent to jo to check
</commit_message>
<xml_diff>
--- a/Dashboard Tracker.xlsx
+++ b/Dashboard Tracker.xlsx
@@ -1040,7 +1040,7 @@
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="L12" s="9" t="inlineStr">
@@ -1367,17 +1367,17 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="K14" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">

</xml_diff>